<commit_message>
cleaned up .lock file
</commit_message>
<xml_diff>
--- a/Birds of the dune.xlsx
+++ b/Birds of the dune.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="140">
   <si>
     <t xml:space="preserve">Name_sc</t>
   </si>
@@ -442,9 +442,6 @@
   </si>
   <si>
     <t xml:space="preserve">Schwalbe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fluss</t>
   </si>
 </sst>
 </file>
@@ -7297,7 +7294,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="B62" s="0" t="n">
         <v>5</v>
@@ -7382,7 +7379,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="B67" s="0" t="n">
         <v>10</v>
@@ -7419,7 +7416,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="B69" s="0" t="n">
         <v>18</v>

</xml_diff>